<commit_message>
Daily scrape output - 2026-09-17
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_odds_data.xlsx
+++ b/outputs/pinnacle_odds_data.xlsx
@@ -555,7 +555,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/sjk-vs-ifk-mariehamn/1636346518</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/fc-lahti-vs-jaro/1636346519</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -570,47 +570,47 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SJK</t>
+          <t>FC Lahti</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Jaro</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-16 10:36</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1.763</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.890</t>
+          <t>4.370</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>4.360</t>
+          <t>5.420</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -623,12 +623,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
@@ -644,7 +644,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/fc-lahti-vs-jaro/1636346519</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/sjk-vs-ifk-mariehamn/1636346518</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -659,47 +659,47 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>SJK</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>IFK Mariehamn</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-16 10:36</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>4.380</t>
+          <t>3.870</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>5.430</t>
+          <t>4.330</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -712,12 +712,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
@@ -758,22 +758,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3.580</t>
+          <t>3.640</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4.120</t>
+          <t>4.290</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -783,12 +783,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -801,12 +801,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
@@ -847,37 +847,37 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2.650</t>
+          <t>2.850</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3.500</t>
+          <t>3.450</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.490</t>
+          <t>2.360</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>2.060</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -890,12 +890,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
@@ -936,7 +936,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -961,12 +961,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -979,12 +979,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
@@ -1000,7 +1000,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/gnistan-vs-hjk-helsinki/1636346549</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/ac-oulu-vs-inter-turku/1636378694</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1015,32 +1015,32 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>AC Oulu</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Inter Turku</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-16 10:36</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3.770</t>
+          <t>4.220</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>4.010</t>
+          <t>3.610</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1063,17 +1063,17 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
@@ -1089,7 +1089,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/ac-oulu-vs-inter-turku/1636378694</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/gnistan-vs-hjk-helsinki/1636346549</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1104,32 +1104,32 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AC Oulu</t>
+          <t>Gnistan</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>HJK Helsinki</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-16 10:36</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4.220</t>
+          <t>3.730</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3.610</t>
+          <t>3.960</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1139,12 +1139,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1152,17 +1152,17 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
@@ -1203,22 +1203,22 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3.990</t>
+          <t>4.120</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3.400</t>
+          <t>3.440</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1228,12 +1228,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1241,17 +1241,17 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
           <t>1.840</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>1.980</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
@@ -1292,17 +1292,17 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2.090</t>
+          <t>2.080</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3.660</t>
+          <t>3.680</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1317,12 +1317,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1335,12 +1335,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:49</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1495,12 +1495,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
@@ -1559,17 +1559,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2.440</t>
+          <t>2.420</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3.530</t>
+          <t>3.560</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1584,12 +1584,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2.080</t>
+          <t>2.090</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1597,17 +1597,17 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
@@ -1623,62 +1623,62 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-bytom-vs-ruch-chorzow/1636382504</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/wisla-krakow-vs-slask-wroclaw/1636378772</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-18 18:45</t>
+          <t>2026-09-18 18:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Polonia Bytom</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2.760</t>
+          <t>1.632</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3.460</t>
+          <t>4.250</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.410</t>
+          <t>4.680</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1686,17 +1686,17 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
@@ -1712,62 +1712,62 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/vila-nova-vs-america-mineiro/1636385547</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-bytom-vs-ruch-chorzow/1636382504</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-18 22:30</t>
+          <t>2026-09-18 18:45</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Vila Nova</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1.483</t>
+          <t>2.760</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>4.150</t>
+          <t>3.480</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>6.760</t>
+          <t>2.410</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1775,17 +1775,17 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
@@ -1801,12 +1801,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/ceara-vs-gremio-novorizontino/1636385559</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/vila-nova-vs-america-mineiro/1636385547</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-18 23:30</t>
+          <t>2026-09-18 22:30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1816,47 +1816,47 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2.900</t>
+          <t>1.456</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3.290</t>
+          <t>4.150</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.460</t>
+          <t>7.400</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2.090</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1864,17 +1864,17 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -1890,12 +1890,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/sao-bernardo-vs-atletico-goianiense/1636385562</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/ceara-vs-gremio-novorizontino/1636385559</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-19 00:00</t>
+          <t>2026-09-18 23:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1905,47 +1905,47 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sao Bernardo</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2.360</t>
+          <t>2.960</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>3.190</t>
+          <t>3.290</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>3.140</t>
+          <t>2.420</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>2.090</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1979,62 +1979,62 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/lechia-gdansk-vs-stal-mielec/1635909038</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/sao-bernardo-vs-atletico-goianiense/1636385562</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-19 10:30</t>
+          <t>2026-09-19 00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Lechia Gdansk</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>2.550</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3.750</t>
+          <t>3.160</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3.240</t>
+          <t>2.890</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2042,17 +2042,17 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -2068,62 +2068,62 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/osters-vs-norrkoping/1636434677</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/lechia-gdansk-vs-stal-mielec/1635909038</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-19 11:00</t>
+          <t>2026-09-19 10:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Lechia Gdansk</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3.940</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4.090</t>
+          <t>3.750</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.757</t>
+          <t>3.240</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>+0.75</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2131,17 +2131,17 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
@@ -2182,22 +2182,22 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2.210</t>
+          <t>2.280</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3.510</t>
+          <t>3.420</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>3.070</t>
+          <t>3.030</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2207,12 +2207,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2225,12 +2225,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -2246,62 +2246,62 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/tps-vs-ilves/1636439257</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/osters-vs-norrkoping/1636434677</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-19 12:00</t>
+          <t>2026-09-19 11:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2.590</t>
+          <t>3.940</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3.670</t>
+          <t>4.090</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2.550</t>
+          <t>1.757</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+0.75</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -2309,17 +2309,17 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2513,7 +2513,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/oddevold-vs-varnamo/1636463784</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/varbergs-bois-vs-brage/1636454979</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2528,47 +2528,47 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2.100</t>
+          <t>1.714</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>3.570</t>
+          <t>3.820</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>3.240</t>
+          <t>4.500</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
@@ -2602,7 +2602,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/varbergs-bois-vs-brage/1636454979</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/oddevold-vs-varnamo/1636463784</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>1.714</t>
+          <t>2.100</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>3.820</t>
+          <t>3.570</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>4.500</t>
+          <t>3.240</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -2670,12 +2670,12 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2869,7 +2869,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-warsaw-vs-chrobry-glogow/1635909036</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/nieciecza-vs-odra-opole/1635909035</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2884,22 +2884,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>4.070</t>
+          <t>3.560</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2919,12 +2919,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -2932,17 +2932,17 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
@@ -2958,7 +2958,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/nieciecza-vs-odra-opole/1635909035</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-warsaw-vs-chrobry-glogow/1635909036</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2973,22 +2973,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Nieciecza</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>3.560</t>
+          <t>4.070</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3008,12 +3008,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -3021,17 +3021,17 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
@@ -3072,7 +3072,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:49</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3695,22 +3695,22 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2.340</t>
+          <t>2.330</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>3.610</t>
+          <t>3.630</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2.850</t>
+          <t>2.860</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3720,12 +3720,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
@@ -3784,37 +3784,37 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2.930</t>
+          <t>3.140</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>3.040</t>
+          <t>3.050</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2.650</t>
+          <t>2.480</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.769</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>2.110</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3873,22 +3873,22 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>1.561</t>
+          <t>1.571</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>4.250</t>
+          <t>4.160</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>5.530</t>
+          <t>5.590</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3898,12 +3898,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -3911,17 +3911,17 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -4051,22 +4051,22 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-16 10:40</t>
+          <t>2026-09-17 10:49</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>1.714</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>3.800</t>
+          <t>3.980</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>4.150</t>
+          <t>4.310</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4076,12 +4076,12 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4407,17 +4407,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2.270</t>
+          <t>2.280</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>2.920</t>
+          <t>2.910</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4585,22 +4585,22 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>3.460</t>
+          <t>3.710</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>3.680</t>
+          <t>3.800</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -4610,12 +4610,12 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="M47" t="inlineStr"/>
@@ -4628,12 +4628,12 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
@@ -4674,17 +4674,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-09-16 10:40</t>
+          <t>2026-09-17 10:49</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>3.250</t>
+          <t>3.280</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>3.580</t>
+          <t>3.560</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="M48" t="inlineStr"/>
@@ -4763,22 +4763,22 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2.430</t>
+          <t>2.450</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>2.990</t>
+          <t>2.970</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>3.300</t>
+          <t>3.280</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -4788,12 +4788,12 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>2.070</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="M49" t="inlineStr"/>
@@ -4806,12 +4806,12 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="S49" t="inlineStr"/>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4941,12 +4941,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2.460</t>
+          <t>2.430</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2.830</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4966,12 +4966,12 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.769</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>2.090</t>
         </is>
       </c>
       <c r="M51" t="inlineStr"/>
@@ -5030,22 +5030,22 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2.100</t>
+          <t>2.110</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>3.670</t>
+          <t>3.640</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>3.190</t>
+          <t>3.200</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5055,12 +5055,12 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="M52" t="inlineStr"/>
@@ -5068,17 +5068,17 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="S52" t="inlineStr"/>
@@ -5119,37 +5119,37 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>9.820</t>
+          <t>9.480</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>5.660</t>
+          <t>5.590</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>1.264</t>
+          <t>1.284</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>+1.75</t>
+          <t>+1.5</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M53" t="inlineStr"/>
@@ -5162,12 +5162,12 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="S53" t="inlineStr"/>
@@ -5208,22 +5208,22 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:46</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2.790</t>
+          <t>2.640</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>3.390</t>
+          <t>3.330</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2.520</t>
+          <t>2.700</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -5233,12 +5233,12 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="M54" t="inlineStr"/>
@@ -5251,12 +5251,12 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="S54" t="inlineStr"/>
@@ -5272,7 +5272,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stabaek-vs-sogndal/1636532662</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/raufoss-vs-stromsgodset/1636498763</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5287,47 +5287,47 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>1.401</t>
+          <t>7.930</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>5.350</t>
+          <t>6.090</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>5.860</t>
+          <t>1.271</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>-1.25</t>
+          <t>+1.75</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="M55" t="inlineStr"/>
@@ -5335,17 +5335,17 @@
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="S55" t="inlineStr"/>
@@ -5361,7 +5361,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/odd-bk-vs-egersunds/1636498750</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/haugesund-vs-strommen/1636498754</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5376,47 +5376,47 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>1.714</t>
+          <t>1.266</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>4.310</t>
+          <t>6.290</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>3.940</t>
+          <t>7.820</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>-1.75</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="M56" t="inlineStr"/>
@@ -5424,17 +5424,17 @@
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S56" t="inlineStr"/>
@@ -5450,7 +5450,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/sandnes-ulf-vs-moss/1636498198</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stabaek-vs-sogndal/1636532662</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -5465,47 +5465,47 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2.170</t>
+          <t>1.400</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>3.800</t>
+          <t>5.360</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2.960</t>
+          <t>5.880</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-1.25</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="M57" t="inlineStr"/>
@@ -5513,7 +5513,7 @@
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="S57" t="inlineStr"/>
@@ -5564,37 +5564,37 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>1.263</t>
+          <t>1.271</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>5.640</t>
+          <t>5.560</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>9.300</t>
+          <t>9.080</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>-2.0</t>
+          <t>-1.75</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="M58" t="inlineStr"/>
@@ -5607,12 +5607,12 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="S58" t="inlineStr"/>
@@ -5628,7 +5628,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/raufoss-vs-stromsgodset/1636498763</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/sandnes-ulf-vs-moss/1636498198</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5643,47 +5643,47 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>7.930</t>
+          <t>2.170</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>6.090</t>
+          <t>3.800</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>1.271</t>
+          <t>2.960</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>+1.75</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="M59" t="inlineStr"/>
@@ -5691,17 +5691,17 @@
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
@@ -5717,7 +5717,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/haugesund-vs-strommen/1636498754</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/odd-bk-vs-egersunds/1636498750</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5732,47 +5732,47 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>1.255</t>
+          <t>1.714</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>6.430</t>
+          <t>4.310</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>8.100</t>
+          <t>3.940</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>-1.75</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="M60" t="inlineStr"/>
@@ -5780,17 +5780,17 @@
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="S60" t="inlineStr"/>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -6073,7 +6073,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/las-palmas-vs-burgos/1636569840</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/almeria-vs-celta-vigo-ii/1636569839</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6088,47 +6088,47 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.393</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>3.020</t>
+          <t>4.910</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>4.450</t>
+          <t>7.360</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>-1.25</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="M64" t="inlineStr"/>
@@ -6136,17 +6136,17 @@
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="S64" t="inlineStr"/>
@@ -6162,7 +6162,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/almeria-vs-celta-vigo-ii/1636569839</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/las-palmas-vs-burgos/1636569840</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -6177,47 +6177,47 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Celta Vigo II</t>
+          <t>Burgos</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>1.377</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>5.050</t>
+          <t>3.020</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>7.480</t>
+          <t>4.390</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>-1.25</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="M65" t="inlineStr"/>
@@ -6225,17 +6225,17 @@
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="S65" t="inlineStr"/>
@@ -6276,22 +6276,22 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-09-16 10:40</t>
+          <t>2026-09-17 10:49</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>1.613</t>
+          <t>1.606</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>4.010</t>
+          <t>4.040</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>5.040</t>
+          <t>5.060</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -6301,12 +6301,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="M66" t="inlineStr"/>
@@ -6319,12 +6319,12 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="S66" t="inlineStr"/>
@@ -6365,22 +6365,22 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>1.280</t>
+          <t>1.290</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>5.900</t>
+          <t>5.790</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>8.370</t>
+          <t>8.160</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -6390,12 +6390,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="M67" t="inlineStr"/>
@@ -6408,12 +6408,12 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S67" t="inlineStr"/>
@@ -6454,7 +6454,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-09-16 10:37</t>
+          <t>2026-09-17 10:47</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -6543,22 +6543,22 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>3.250</t>
+          <t>3.260</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>4.590</t>
+          <t>4.630</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -6568,12 +6568,12 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="M69" t="inlineStr"/>
@@ -6586,12 +6586,12 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="S69" t="inlineStr"/>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -6696,12 +6696,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/petrolul-ploiesti-vs-csikszereda/1636618551</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/otelul-galati-vs-corvinul-hunedoara/1636611974</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-09-21 18:00</t>
+          <t>2026-09-21 15:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -6711,47 +6711,47 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-09-16 10:40</t>
+          <t>2026-09-17 10:49</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>1.680</t>
+          <t>2.420</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>3.710</t>
+          <t>3.130</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>4.930</t>
+          <t>3.070</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>2.060</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.769</t>
         </is>
       </c>
       <c r="M71" t="inlineStr"/>
@@ -6759,17 +6759,17 @@
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="S71" t="inlineStr"/>
@@ -6785,42 +6785,42 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/criciuma-vs-operario-ferroviario/1636636585</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/petrolul-ploiesti-vs-csikszereda/1636618551</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-09-21 22:30</t>
+          <t>2026-09-21 18:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Petrolul Ploiesti</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Csikszereda</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-09-16 10:38</t>
+          <t>2026-09-17 10:49</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.680</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>3.380</t>
+          <t>3.710</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6835,12 +6835,12 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="M72" t="inlineStr"/>
@@ -6848,17 +6848,17 @@
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="S72" t="inlineStr"/>
@@ -6874,12 +6874,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/cuiaba-vs-nautico/1636640777</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/criciuma-vs-operario-ferroviario/1636636585</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-09-22 00:30</t>
+          <t>2026-09-21 22:30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6889,47 +6889,47 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-09-16 10:39</t>
+          <t>2026-09-17 10:48</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2.090</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>3.210</t>
+          <t>3.380</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>3.770</t>
+          <t>4.930</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>2.070</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="M73" t="inlineStr"/>
@@ -6942,12 +6942,12 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="S73" t="inlineStr"/>
@@ -6960,6 +6960,95 @@
       <c r="Z73" t="inlineStr"/>
       <c r="AA73" t="inlineStr"/>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/cuiaba-vs-nautico/1636640777</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-09-22 00:30</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:48</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2.050</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>3.240</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>3.860</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>2.060</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>1.793</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>1.826</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="inlineStr"/>
+      <c r="W74" t="inlineStr"/>
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr"/>
+      <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-03
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_odds_data.xlsx
+++ b/outputs/pinnacle_odds_data.xlsx
@@ -552,6 +552,718 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/wieczysta-krakow-vs-wisla-plock/1637178773</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Wieczysta Krakow</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:54</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2.160</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3.600</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>3.180</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1.980</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/galatasaray-vs-kasimpasa/1637175572</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kasimpasa</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:55</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1.234</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>6.330</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>10.640</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>-1.75</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1.854</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/moreirense-vs-gil-vicente/1637175573</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:45</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Moreirense</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:56</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3.600</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3.100</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2.230</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>+0.25</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1.892</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2.070</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1.787</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/rakow-czestochowa-vs-gks-katowice/1637178774</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:30</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:55</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2.170</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>3.950</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2.920</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1.909</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1.833</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/podbeskidzie-bielsko-biala-vs-pogon-siedlce/1637352530</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Podbeskidzie Bielsko-Biala</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:55</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1.769</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>3.690</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>4.250</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-0.75</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2.020</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1.800</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1.826</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/borussia-dortmund-vs-werder-bremen/1636598006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:55</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1.400</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>5.430</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>6.850</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>-1.5</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2.010</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1.877</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1.869</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/braga-vs-sporting-cp/1637181731</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-09 19:15</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:57</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>3.410</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>3.440</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2.140</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>+0.25</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1.854</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1.990</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1.854</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/genclerbirligi-vs-amedspor/1637178745</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Genclerbirligi</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Amedspor</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:55</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2.590</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>3.520</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2.310</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1.740</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1.892</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1.787</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-04
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_odds_data.xlsx
+++ b/outputs/pinnacle_odds_data.xlsx
@@ -580,7 +580,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-10-03 10:54</t>
+          <t>2026-10-04 11:37</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -669,22 +669,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-03 10:55</t>
+          <t>2026-10-04 11:37</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.234</t>
+          <t>1.238</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>6.330</t>
+          <t>6.260</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>10.640</t>
+          <t>10.520</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -712,12 +712,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
@@ -758,7 +758,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-10-03 10:56</t>
+          <t>2026-10-04 11:38</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-03 10:55</t>
+          <t>2026-10-04 11:37</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-03 10:55</t>
+          <t>2026-10-04 11:37</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1025,22 +1025,22 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-10-03 10:55</t>
+          <t>2026-10-04 11:38</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1.400</t>
+          <t>1.409</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>5.430</t>
+          <t>5.420</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>6.850</t>
+          <t>6.890</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1068,12 +1068,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-03 10:57</t>
+          <t>2026-10-04 11:38</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-10-03 10:55</t>
+          <t>2026-10-04 11:37</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1264,6 +1264,1697 @@
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/cracovia-krakow-vs-zaglebie-lubin/1637178775</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-10 12:45</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1.900</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>3.430</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>4.180</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1.909</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1.892</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/samsunspor-vs-trabzonspor/1637178747</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Samsunspor</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3.460</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>3.650</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2.050</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>+0.5</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>1.806</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2.060</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1.990</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/alanyaspor-vs-erzurumspor/1637178748</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Alanyaspor</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Erzurumspor</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1.943</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>3.120</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3.700</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1.751</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1.900</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1.781</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/arka-gdynia-vs-polonia-warsaw/1637398417</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Arka Gdynia</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2.270</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3.480</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2.960</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>1.980</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1.833</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1.813</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1.980</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/unia-skierniewice-vs-nieciecza/1637396143</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Unia Skierniewice</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Nieciecza</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2.580</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>3.660</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2.470</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>1.943</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1.862</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1.900</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/chrobry-glogow-vs-pogon-grodzisk-mazowiecki/1637397488</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2.180</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>3.460</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>3.130</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>1.900</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>1.900</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1.840</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/union-berlin-vs-elversberg/1636598008</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2.300</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>3.980</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2.840</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2.030</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1.862</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1.934</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1.934</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/hoffenheim-vs-hamburger-sv/1636590116</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1.436</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>4.860</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>7.010</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>-1.25</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2.030</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/mainz-05-vs-bayer-leverkusen/1636598004</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mainz 05</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2.960</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>3.960</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2.230</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>+0.25</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1.970</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1.943</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/paderborn-vs-stuttgart/1636592221</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4.820</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>4.680</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1.606</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>+1.0</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1.970</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1.877</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/augsburg-vs-bayern-munich/1636592218</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:30</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>8.930</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>8.680</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1.215</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>+2.25</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>1.877</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1.970</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1.877</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/casa-pia-vs-santa-clara/1637175574</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-10-10 14:30</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Casa Pia</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Santa Clara</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4.300</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>3.370</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1.909</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>+0.5</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>1.934</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1.781</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>2.080</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/slask-wroclaw-vs-lech-poznan/1637360367</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Slask Wroclaw</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4.900</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>4.480</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1.574</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>+1.0</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>1.877</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1.826</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/caykur-rizespor-vs-fenerbahce/1637178749</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:00</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Fenerbahce</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4.370</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>4.030</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1.735</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>+0.75</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>1.934</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1.819</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>2.030</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/rb-leipzig-vs-eintracht-frankfurt/1636592222</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:30</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1.543</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>4.990</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>5.110</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>-1.0</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2.050</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>3.75</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/jagiellonia-bialystok-vs-gornik-zabrze/1637183910</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-10 18:15</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2.550</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>3.410</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2.710</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>1.854</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>1.980</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1.892</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/academico-de-viseu-vs-estoril/1637175575</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-10 19:30</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Academico de Viseu</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2.290</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>3.380</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>3.150</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>1.980</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>1.877</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/stal-mielec-vs-warta-poznan/1637426540</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-11 10:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Warta Poznan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:37</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2.920</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>3.750</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2.190</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>+0.25</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1.869</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1.862</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/konyaspor-vs-istanbul-basaksehir/1637181716</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-11 10:30</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Konyaspor</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-10-04 11:38</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2.570</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>3.420</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2.720</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>1.877</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>1.980</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>2.010</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1.833</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-05
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_odds_data.xlsx
+++ b/outputs/pinnacle_odds_data.xlsx
@@ -580,7 +580,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:13</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -733,62 +733,62 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/moreirense-vs-gil-vicente/1637175573</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/rakow-czestochowa-vs-gks-katowice/1637178774</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-09 17:45</t>
+          <t>2026-10-09 18:30</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Moreirense</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:13</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3.600</t>
+          <t>2.170</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3.100</t>
+          <t>3.950</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2.230</t>
+          <t>2.920</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -796,17 +796,17 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.070</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
@@ -822,7 +822,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/rakow-czestochowa-vs-gks-katowice/1637178774</t>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/borussia-dortmund-vs-werder-bremen/1636598006</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -832,52 +832,52 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>Borussia Dortmund</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>Werder Bremen</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2.170</t>
+          <t>1.403</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3.950</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.920</t>
+          <t>6.970</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-1.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -885,17 +885,17 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
@@ -911,62 +911,62 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/podbeskidzie-bielsko-biala-vs-pogon-siedlce/1637352530</t>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/braga-vs-sporting-cp/1637181731</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-09 18:30</t>
+          <t>2026-10-09 19:15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Podbeskidzie Bielsko-Biala</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Sporting CP</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:15</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>3.610</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3.690</t>
+          <t>3.470</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>4.250</t>
+          <t>2.060</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>+0.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>2.070</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -979,12 +979,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
@@ -1000,62 +1000,62 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/borussia-dortmund-vs-werder-bremen/1636598006</t>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/genclerbirligi-vs-amedspor/1637178745</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-09 18:30</t>
+          <t>2026-10-10 10:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Borussia Dortmund</t>
+          <t>Genclerbirligi</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Werder Bremen</t>
+          <t>Amedspor</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1.409</t>
+          <t>2.370</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>5.420</t>
+          <t>3.520</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>6.890</t>
+          <t>2.520</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-1.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1063,17 +1063,17 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
@@ -1089,62 +1089,62 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/braga-vs-sporting-cp/1637181731</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/cracovia-krakow-vs-zaglebie-lubin/1637178775</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-09 19:15</t>
+          <t>2026-10-10 12:45</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sporting CP</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:13</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3.410</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3.440</t>
+          <t>3.430</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2.140</t>
+          <t>4.180</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
@@ -1178,12 +1178,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/genclerbirligi-vs-amedspor/1637178745</t>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/samsunspor-vs-trabzonspor/1637178747</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30</t>
+          <t>2026-10-10 13:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1193,47 +1193,47 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Genclerbirligi</t>
+          <t>Samsunspor</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Amedspor</t>
+          <t>Trabzonspor</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.590</t>
+          <t>3.460</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3.520</t>
+          <t>3.650</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2.310</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+0.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1.740</t>
+          <t>2.060</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1246,12 +1246,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
@@ -1267,47 +1267,47 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/cracovia-krakow-vs-zaglebie-lubin/1637178775</t>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/alanyaspor-vs-erzurumspor/1637178748</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-10 12:45</t>
+          <t>2026-10-10 13:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Erzurumspor</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3.430</t>
+          <t>3.120</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>4.180</t>
+          <t>3.700</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1317,12 +1317,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.751</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1330,17 +1330,17 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
@@ -1356,62 +1356,62 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/samsunspor-vs-trabzonspor/1637178747</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/unia-skierniewice-vs-nieciecza/1637396143</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-10 13:00</t>
+          <t>2026-10-10 13:30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Samsunspor</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3.460</t>
+          <t>2.580</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3.650</t>
+          <t>3.660</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>2.470</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1419,17 +1419,17 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
@@ -1445,62 +1445,62 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/alanyaspor-vs-erzurumspor/1637178748</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/arka-gdynia-vs-polonia-warsaw/1637398417</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-10 13:00</t>
+          <t>2026-10-10 13:30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Alanyaspor</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Erzurumspor</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>2.270</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3.120</t>
+          <t>3.480</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3.700</t>
+          <t>2.960</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.751</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1508,17 +1508,17 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
@@ -1534,7 +1534,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/arka-gdynia-vs-polonia-warsaw/1637398417</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/chrobry-glogow-vs-pogon-grodzisk-mazowiecki/1637397488</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1549,32 +1549,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Arka Gdynia</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2.270</t>
+          <t>2.180</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3.480</t>
+          <t>3.460</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2.960</t>
+          <t>3.130</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1584,12 +1584,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1597,17 +1597,17 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
@@ -1623,7 +1623,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/unia-skierniewice-vs-nieciecza/1637396143</t>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/augsburg-vs-bayern-munich/1636592218</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1633,52 +1633,52 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Unia Skierniewice</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Nieciecza</t>
+          <t>Bayern Munich</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2.580</t>
+          <t>9.500</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3.660</t>
+          <t>9.030</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.470</t>
+          <t>1.208</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+2.25</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1686,17 +1686,17 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
@@ -1712,7 +1712,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/chrobry-glogow-vs-pogon-grodzisk-mazowiecki/1637397488</t>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/paderborn-vs-stuttgart/1636592221</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1722,52 +1722,52 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Paderborn</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2.180</t>
+          <t>4.840</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3.460</t>
+          <t>4.710</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3.130</t>
+          <t>1.617</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>+1.0</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1775,17 +1775,17 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
@@ -1801,7 +1801,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/union-berlin-vs-elversberg/1636598008</t>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/mainz-05-vs-bayer-leverkusen/1636598004</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1816,47 +1816,47 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Union Berlin</t>
+          <t>Mainz 05</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Bayer Leverkusen</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2.300</t>
+          <t>3.000</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3.980</t>
+          <t>3.990</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.840</t>
+          <t>2.220</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1864,7 +1864,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -1915,22 +1915,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>1.436</t>
+          <t>1.442</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4.860</t>
+          <t>4.900</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>7.010</t>
+          <t>7.090</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1940,12 +1940,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -1958,12 +1958,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
@@ -1979,7 +1979,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/mainz-05-vs-bayer-leverkusen/1636598004</t>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/union-berlin-vs-elversberg/1636598008</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1994,47 +1994,47 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mainz 05</t>
+          <t>Union Berlin</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2.960</t>
+          <t>2.330</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3.960</t>
+          <t>3.900</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2.230</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2042,17 +2042,17 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -2068,62 +2068,62 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/paderborn-vs-stuttgart/1636592221</t>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/casa-pia-vs-santa-clara/1637175574</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-10 13:30</t>
+          <t>2026-10-10 14:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paderborn</t>
+          <t>Casa Pia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:15</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4.820</t>
+          <t>4.300</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4.680</t>
+          <t>3.370</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.606</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>+1.0</t>
+          <t>+0.5</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
+          <t>1.934</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
           <t>1.917</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>1.970</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2131,17 +2131,17 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>2.080</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
@@ -2157,52 +2157,52 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/augsburg-vs-bayern-munich/1636592218</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/slask-wroclaw-vs-lech-poznan/1637360367</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-10 13:30</t>
+          <t>2026-10-10 15:30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:13</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8.930</t>
+          <t>4.900</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>8.680</t>
+          <t>4.480</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1.215</t>
+          <t>1.574</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>+2.25</t>
+          <t>+1.0</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2220,17 +2220,17 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -2246,62 +2246,62 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/casa-pia-vs-santa-clara/1637175574</t>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/caykur-rizespor-vs-fenerbahce/1637178749</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-10 14:30</t>
+          <t>2026-10-10 16:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Caykur Rizespor</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>Fenerbahce</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>4.300</t>
+          <t>4.370</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3.370</t>
+          <t>4.030</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.735</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>+0.75</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
           <t>1.934</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>1.917</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -2309,17 +2309,17 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>2.080</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -2335,62 +2335,62 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/slask-wroclaw-vs-lech-poznan/1637360367</t>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/rb-leipzig-vs-eintracht-frankfurt/1636592222</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-10 15:30</t>
+          <t>2026-10-10 16:30</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Slask Wroclaw</t>
+          <t>RB Leipzig</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4.900</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>4.480</t>
+          <t>4.990</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.574</t>
+          <t>5.150</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>+1.0</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -2398,7 +2398,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
@@ -2424,62 +2424,62 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/caykur-rizespor-vs-fenerbahce/1637178749</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/jagiellonia-bialystok-vs-gornik-zabrze/1637183910</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-10 16:00</t>
+          <t>2026-10-10 18:15</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Caykur Rizespor</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fenerbahce</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:13</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4.370</t>
+          <t>2.550</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>4.030</t>
+          <t>3.410</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1.735</t>
+          <t>2.710</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>+0.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -2492,12 +2492,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
@@ -2513,62 +2513,62 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/rb-leipzig-vs-eintracht-frankfurt/1636592222</t>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/academico-de-viseu-vs-estoril/1637175575</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-10 16:30</t>
+          <t>2026-10-10 19:30</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Academico de Viseu</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:15</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>1.543</t>
+          <t>2.290</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4.990</t>
+          <t>3.380</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>5.110</t>
+          <t>3.150</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -2576,12 +2576,12 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2602,62 +2602,62 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/jagiellonia-bialystok-vs-gornik-zabrze/1637183910</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/stal-mielec-vs-warta-poznan/1637426540</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-10 18:15</t>
+          <t>2026-10-11 10:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Warta Poznan</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2.550</t>
+          <t>2.760</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>3.410</t>
+          <t>3.680</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2.710</t>
+          <t>2.320</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -2665,17 +2665,17 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
@@ -2691,62 +2691,62 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/academico-de-viseu-vs-estoril/1637175575</t>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/konyaspor-vs-istanbul-basaksehir/1637181716</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-10 19:30</t>
+          <t>2026-10-11 10:30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Academico de Viseu</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Istanbul Basaksehir</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2.290</t>
+          <t>2.710</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>3.380</t>
+          <t>3.350</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>3.150</t>
+          <t>2.620</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -2759,12 +2759,12 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
@@ -2780,12 +2780,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/stal-mielec-vs-warta-poznan/1637426540</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/lks-lodz-vs-ruch-chorzow/1637429081</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-11 10:00</t>
+          <t>2026-10-11 12:30</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2795,47 +2795,47 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Warta Poznan</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-10-04 11:37</t>
+          <t>2026-10-05 13:14</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2.920</t>
+          <t>2.440</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3.750</t>
+          <t>3.380</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2.190</t>
+          <t>2.780</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2843,17 +2843,17 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
@@ -2869,47 +2869,47 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/konyaspor-vs-istanbul-basaksehir/1637181716</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/piast-gliwice-vs-widzew-lodz/1637181739</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-11 10:30</t>
+          <t>2026-10-11 12:45</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Konyaspor</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-10-04 11:38</t>
+          <t>2026-10-05 13:13</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2.570</t>
+          <t>2.690</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>3.420</t>
+          <t>3.490</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2.720</t>
+          <t>2.530</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2919,12 +2919,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -2937,12 +2937,12 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
@@ -2955,6 +2955,896 @@
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/gaziantep-vs-corum-belediyespor/1637175580</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-11 13:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Gaziantep</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Corum Belediyespor</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:14</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2.700</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>3.340</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2.630</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>1.900</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1.862</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1.970</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/fc-koln-vs-borussia-monchengladbach/1636598005</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-11 13:30</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>FC Koln</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Borussia Monchengladbach</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:14</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2.030</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>4.150</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>3.260</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>2.040</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>1.854</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1.869</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/rio-ave-vs-nacional-da-madeira/1637175576</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-10-11 14:30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Rio Ave</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Nacional da Madeira</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:15</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2.340</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>3.250</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>3.190</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2.010</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1.833</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>2.010</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/puszcza-niepolomice-vs-polonia-bytom/1637432116</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:14</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2.470</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>3.720</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2.550</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>1.869</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>1.934</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1.990</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1.800</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/pogon-szczecin-vs-korona-kielce/1637178776</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:30</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:13</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2.290</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>3.080</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>3.390</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1.970</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/germany-bundesliga/freiburg-vs-schalke-04/1636590120</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:30</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:14</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>1.666</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>3.930</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>5.280</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>-0.75</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2.050</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>2.030</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/turkey-super-league/besiktas-vs-kocaelispor/1637181718</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-10-11 16:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Kocaelispor</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:14</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>1.261</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>5.800</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>10.270</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>-1.75</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2.010</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>1.833</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1.970</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/legia-warsaw-vs-wisla-krakow/1637183911</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-10-11 18:15</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Wisla Krakow</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:13</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>1.990</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>3.840</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>3.410</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>1.847</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>2.030</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1.800</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/odra-opole-vs-miedz-legnica/1637436570</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-10-11 18:15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:14</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2.440</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>3.420</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2.750</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>1.793</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2.020</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1.990</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1.806</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>https://www.pinnacle.com/en/soccer/portugal-primeira-liga/arouca-vs-estrela-da-amadora/1637181732</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-10-11 19:30</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Arouca</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Estrela da Amadora</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:16</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2.170</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>3.530</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>3.250</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>1.892</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1.909</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1.925</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>